<commit_message>
début d'ajout de la méthode avec le point deja présent et petit refactoring de classes.py et main.py
</commit_message>
<xml_diff>
--- a/ListPoint.xlsx
+++ b/ListPoint.xlsx
@@ -262,7 +262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C421"/>
+  <dimension ref="A1:C793"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -4347,553 +4347,4645 @@
       </c>
     </row>
     <row r="372">
-      <c r="A372" t="n">
+      <c r="A372" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B372" t="n">
+      <c r="B372" s="0" t="n">
         <v>643</v>
       </c>
-      <c r="C372" t="n">
+      <c r="C372" s="0" t="n">
         <v>424</v>
       </c>
     </row>
     <row r="373">
-      <c r="A373" t="n">
+      <c r="A373" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B373" t="n">
+      <c r="B373" s="0" t="n">
         <v>1165</v>
       </c>
-      <c r="C373" t="n">
+      <c r="C373" s="0" t="n">
         <v>446</v>
       </c>
     </row>
     <row r="374">
-      <c r="A374" t="n">
+      <c r="A374" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B374" t="n">
+      <c r="B374" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C374" t="n">
+      <c r="C374" s="0" t="n">
         <v>680</v>
       </c>
     </row>
     <row r="375">
-      <c r="A375" t="n">
+      <c r="A375" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B375" t="n">
+      <c r="B375" s="0" t="n">
         <v>107</v>
       </c>
-      <c r="C375" t="n">
+      <c r="C375" s="0" t="n">
         <v>161</v>
       </c>
     </row>
     <row r="376">
-      <c r="A376" t="n">
+      <c r="A376" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B376" t="n">
+      <c r="B376" s="0" t="n">
         <v>989</v>
       </c>
-      <c r="C376" t="n">
+      <c r="C376" s="0" t="n">
         <v>440</v>
       </c>
     </row>
     <row r="377">
-      <c r="A377" t="n">
+      <c r="A377" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B377" t="n">
+      <c r="B377" s="0" t="n">
         <v>957</v>
       </c>
-      <c r="C377" t="n">
+      <c r="C377" s="0" t="n">
         <v>84</v>
       </c>
     </row>
     <row r="378">
-      <c r="A378" t="n">
+      <c r="A378" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B378" t="n">
+      <c r="B378" s="0" t="n">
         <v>441</v>
       </c>
-      <c r="C378" t="n">
+      <c r="C378" s="0" t="n">
         <v>157</v>
       </c>
     </row>
     <row r="379">
-      <c r="A379" t="n">
+      <c r="A379" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B379" t="n">
+      <c r="B379" s="0" t="n">
         <v>801</v>
       </c>
-      <c r="C379" t="n">
+      <c r="C379" s="0" t="n">
         <v>128</v>
       </c>
     </row>
     <row r="380">
-      <c r="A380" t="n">
+      <c r="A380" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B380" t="n">
+      <c r="B380" s="0" t="n">
         <v>215</v>
       </c>
-      <c r="C380" t="n">
+      <c r="C380" s="0" t="n">
         <v>360</v>
       </c>
     </row>
     <row r="381">
-      <c r="A381" t="n">
+      <c r="A381" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B381" t="n">
+      <c r="B381" s="0" t="n">
         <v>737</v>
       </c>
-      <c r="C381" t="n">
+      <c r="C381" s="0" t="n">
         <v>449</v>
       </c>
     </row>
     <row r="382">
-      <c r="A382" t="n">
+      <c r="A382" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B382" t="n">
+      <c r="B382" s="0" t="n">
         <v>261</v>
       </c>
-      <c r="C382" t="n">
+      <c r="C382" s="0" t="n">
         <v>354</v>
       </c>
     </row>
     <row r="383">
-      <c r="A383" t="n">
+      <c r="A383" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B383" t="n">
+      <c r="B383" s="0" t="n">
         <v>479</v>
       </c>
-      <c r="C383" t="n">
+      <c r="C383" s="0" t="n">
         <v>433</v>
       </c>
     </row>
     <row r="384">
-      <c r="A384" t="n">
+      <c r="A384" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B384" t="n">
+      <c r="B384" s="0" t="n">
         <v>1180</v>
       </c>
-      <c r="C384" t="n">
+      <c r="C384" s="0" t="n">
         <v>494</v>
       </c>
     </row>
     <row r="385">
-      <c r="A385" t="n">
+      <c r="A385" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B385" t="n">
+      <c r="B385" s="0" t="n">
         <v>1198</v>
       </c>
-      <c r="C385" t="n">
+      <c r="C385" s="0" t="n">
         <v>77</v>
       </c>
     </row>
     <row r="386">
-      <c r="A386" t="n">
+      <c r="A386" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B386" t="n">
+      <c r="B386" s="0" t="n">
         <v>619</v>
       </c>
-      <c r="C386" t="n">
+      <c r="C386" s="0" t="n">
         <v>95</v>
       </c>
     </row>
     <row r="387">
-      <c r="A387" t="n">
+      <c r="A387" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B387" t="n">
+      <c r="B387" s="0" t="n">
         <v>691</v>
       </c>
-      <c r="C387" t="n">
+      <c r="C387" s="0" t="n">
         <v>257</v>
       </c>
     </row>
     <row r="388">
-      <c r="A388" t="n">
+      <c r="A388" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B388" t="n">
+      <c r="B388" s="0" t="n">
         <v>1186</v>
       </c>
-      <c r="C388" t="n">
+      <c r="C388" s="0" t="n">
         <v>796</v>
       </c>
     </row>
     <row r="389">
-      <c r="A389" t="n">
+      <c r="A389" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B389" t="n">
+      <c r="B389" s="0" t="n">
         <v>1057</v>
       </c>
-      <c r="C389" t="n">
+      <c r="C389" s="0" t="n">
         <v>825</v>
       </c>
     </row>
     <row r="390">
-      <c r="A390" t="n">
+      <c r="A390" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B390" t="n">
+      <c r="B390" s="0" t="n">
         <v>288</v>
       </c>
-      <c r="C390" t="n">
+      <c r="C390" s="0" t="n">
         <v>392</v>
       </c>
     </row>
     <row r="391">
-      <c r="A391" t="n">
+      <c r="A391" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B391" t="n">
+      <c r="B391" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C391" t="n">
+      <c r="C391" s="0" t="n">
         <v>165</v>
       </c>
     </row>
     <row r="392">
-      <c r="A392" t="n">
+      <c r="A392" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B392" t="n">
+      <c r="B392" s="0" t="n">
         <v>63</v>
       </c>
-      <c r="C392" t="n">
+      <c r="C392" s="0" t="n">
         <v>442</v>
       </c>
     </row>
     <row r="393">
-      <c r="A393" t="n">
+      <c r="A393" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B393" t="n">
+      <c r="B393" s="0" t="n">
         <v>657</v>
       </c>
-      <c r="C393" t="n">
+      <c r="C393" s="0" t="n">
         <v>208</v>
       </c>
     </row>
     <row r="394">
-      <c r="A394" t="n">
+      <c r="A394" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B394" t="n">
+      <c r="B394" s="0" t="n">
         <v>486</v>
       </c>
-      <c r="C394" t="n">
+      <c r="C394" s="0" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="395">
-      <c r="A395" t="n">
+      <c r="A395" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B395" t="n">
+      <c r="B395" s="0" t="n">
         <v>697</v>
       </c>
-      <c r="C395" t="n">
+      <c r="C395" s="0" t="n">
         <v>597</v>
       </c>
     </row>
     <row r="396">
-      <c r="A396" t="n">
+      <c r="A396" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B396" t="n">
+      <c r="B396" s="0" t="n">
         <v>439</v>
       </c>
-      <c r="C396" t="n">
+      <c r="C396" s="0" t="n">
         <v>417</v>
       </c>
     </row>
     <row r="397">
-      <c r="A397" t="n">
+      <c r="A397" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B397" t="n">
+      <c r="B397" s="0" t="n">
         <v>879</v>
       </c>
-      <c r="C397" t="n">
+      <c r="C397" s="0" t="n">
         <v>859</v>
       </c>
     </row>
     <row r="398">
-      <c r="A398" t="n">
+      <c r="A398" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B398" t="n">
+      <c r="B398" s="0" t="n">
         <v>416</v>
       </c>
-      <c r="C398" t="n">
+      <c r="C398" s="0" t="n">
         <v>247</v>
       </c>
     </row>
     <row r="399">
-      <c r="A399" t="n">
+      <c r="A399" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B399" t="n">
+      <c r="B399" s="0" t="n">
         <v>1083</v>
       </c>
-      <c r="C399" t="n">
+      <c r="C399" s="0" t="n">
         <v>236</v>
       </c>
     </row>
     <row r="400">
-      <c r="A400" t="n">
+      <c r="A400" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B400" t="n">
+      <c r="B400" s="0" t="n">
         <v>939</v>
       </c>
-      <c r="C400" t="n">
+      <c r="C400" s="0" t="n">
         <v>375</v>
       </c>
     </row>
     <row r="401">
-      <c r="A401" t="n">
+      <c r="A401" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B401" t="n">
+      <c r="B401" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="C401" t="n">
+      <c r="C401" s="0" t="n">
         <v>188</v>
       </c>
     </row>
     <row r="402">
-      <c r="A402" t="n">
+      <c r="A402" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B402" t="n">
+      <c r="B402" s="0" t="n">
         <v>1112</v>
       </c>
-      <c r="C402" t="n">
+      <c r="C402" s="0" t="n">
         <v>239</v>
       </c>
     </row>
     <row r="403">
-      <c r="A403" t="n">
+      <c r="A403" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B403" t="n">
+      <c r="B403" s="0" t="n">
         <v>165</v>
       </c>
-      <c r="C403" t="n">
+      <c r="C403" s="0" t="n">
         <v>890</v>
       </c>
     </row>
     <row r="404">
-      <c r="A404" t="n">
+      <c r="A404" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B404" t="n">
+      <c r="B404" s="0" t="n">
         <v>809</v>
       </c>
-      <c r="C404" t="n">
+      <c r="C404" s="0" t="n">
         <v>467</v>
       </c>
     </row>
     <row r="405">
-      <c r="A405" t="n">
+      <c r="A405" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B405" t="n">
+      <c r="B405" s="0" t="n">
         <v>1192</v>
       </c>
-      <c r="C405" t="n">
+      <c r="C405" s="0" t="n">
         <v>591</v>
       </c>
     </row>
     <row r="406">
-      <c r="A406" t="n">
+      <c r="A406" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B406" t="n">
+      <c r="B406" s="0" t="n">
         <v>879</v>
       </c>
-      <c r="C406" t="n">
+      <c r="C406" s="0" t="n">
         <v>425</v>
       </c>
     </row>
     <row r="407">
-      <c r="A407" t="n">
+      <c r="A407" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B407" t="n">
+      <c r="B407" s="0" t="n">
         <v>913</v>
       </c>
-      <c r="C407" t="n">
+      <c r="C407" s="0" t="n">
         <v>331</v>
       </c>
     </row>
     <row r="408">
-      <c r="A408" t="n">
+      <c r="A408" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B408" t="n">
+      <c r="B408" s="0" t="n">
         <v>1070</v>
       </c>
-      <c r="C408" t="n">
+      <c r="C408" s="0" t="n">
         <v>721</v>
       </c>
     </row>
     <row r="409">
-      <c r="A409" t="n">
+      <c r="A409" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B409" t="n">
+      <c r="B409" s="0" t="n">
         <v>1015</v>
       </c>
-      <c r="C409" t="n">
+      <c r="C409" s="0" t="n">
         <v>780</v>
       </c>
     </row>
     <row r="410">
-      <c r="A410" t="n">
+      <c r="A410" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B410" t="n">
+      <c r="B410" s="0" t="n">
         <v>334</v>
       </c>
-      <c r="C410" t="n">
+      <c r="C410" s="0" t="n">
         <v>692</v>
       </c>
     </row>
     <row r="411">
-      <c r="A411" t="n">
+      <c r="A411" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B411" t="n">
+      <c r="B411" s="0" t="n">
         <v>633</v>
       </c>
-      <c r="C411" t="n">
+      <c r="C411" s="0" t="n">
         <v>92</v>
       </c>
     </row>
     <row r="412">
-      <c r="A412" t="n">
+      <c r="A412" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B412" t="n">
+      <c r="B412" s="0" t="n">
         <v>1136</v>
       </c>
-      <c r="C412" t="n">
+      <c r="C412" s="0" t="n">
         <v>710</v>
       </c>
     </row>
     <row r="413">
-      <c r="A413" t="n">
+      <c r="A413" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B413" t="n">
+      <c r="B413" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="C413" t="n">
+      <c r="C413" s="0" t="n">
         <v>666</v>
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="n">
+      <c r="A414" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B414" t="n">
+      <c r="B414" s="0" t="n">
         <v>583</v>
       </c>
-      <c r="C414" t="n">
+      <c r="C414" s="0" t="n">
         <v>388</v>
       </c>
     </row>
     <row r="415">
-      <c r="A415" t="n">
+      <c r="A415" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B415" t="n">
+      <c r="B415" s="0" t="n">
         <v>686</v>
       </c>
-      <c r="C415" t="n">
+      <c r="C415" s="0" t="n">
         <v>670</v>
       </c>
     </row>
     <row r="416">
-      <c r="A416" t="n">
+      <c r="A416" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B416" t="n">
+      <c r="B416" s="0" t="n">
         <v>621</v>
       </c>
-      <c r="C416" t="n">
+      <c r="C416" s="0" t="n">
         <v>457</v>
       </c>
     </row>
     <row r="417">
-      <c r="A417" t="n">
+      <c r="A417" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B417" t="n">
+      <c r="B417" s="0" t="n">
         <v>696</v>
       </c>
-      <c r="C417" t="n">
+      <c r="C417" s="0" t="n">
         <v>216</v>
       </c>
     </row>
     <row r="418">
-      <c r="A418" t="n">
+      <c r="A418" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B418" t="n">
+      <c r="B418" s="0" t="n">
         <v>834</v>
       </c>
-      <c r="C418" t="n">
+      <c r="C418" s="0" t="n">
         <v>876</v>
       </c>
     </row>
     <row r="419">
-      <c r="A419" t="n">
+      <c r="A419" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B419" t="n">
+      <c r="B419" s="0" t="n">
         <v>905</v>
       </c>
-      <c r="C419" t="n">
+      <c r="C419" s="0" t="n">
         <v>126</v>
       </c>
     </row>
     <row r="420">
-      <c r="A420" t="n">
+      <c r="A420" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B420" t="n">
+      <c r="B420" s="0" t="n">
         <v>417</v>
       </c>
-      <c r="C420" t="n">
+      <c r="C420" s="0" t="n">
         <v>750</v>
       </c>
     </row>
     <row r="421">
-      <c r="A421" t="n">
+      <c r="A421" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B421" t="n">
+      <c r="B421" s="0" t="n">
         <v>1099</v>
       </c>
-      <c r="C421" t="n">
+      <c r="C421" s="0" t="n">
         <v>245</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B422" s="0" t="n">
+        <v>885</v>
+      </c>
+      <c r="C422" s="0" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B423" s="0" t="n">
+        <v>419</v>
+      </c>
+      <c r="C423" s="0" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B424" s="0" t="n">
+        <v>482</v>
+      </c>
+      <c r="C424" s="0" t="n">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B425" s="0" t="n">
+        <v>466</v>
+      </c>
+      <c r="C425" s="0" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B426" s="0" t="n">
+        <v>297</v>
+      </c>
+      <c r="C426" s="0" t="n">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B427" s="0" t="n">
+        <v>482</v>
+      </c>
+      <c r="C427" s="0" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B428" s="0" t="n">
+        <v>278</v>
+      </c>
+      <c r="C428" s="0" t="n">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B429" s="0" t="n">
+        <v>1102</v>
+      </c>
+      <c r="C429" s="0" t="n">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B430" s="0" t="n">
+        <v>959</v>
+      </c>
+      <c r="C430" s="0" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B431" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="C431" s="0" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B432" s="0" t="n">
+        <v>1142</v>
+      </c>
+      <c r="C432" s="0" t="n">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B433" s="0" t="n">
+        <v>531</v>
+      </c>
+      <c r="C433" s="0" t="n">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B434" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C434" s="0" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B435" s="0" t="n">
+        <v>433</v>
+      </c>
+      <c r="C435" s="0" t="n">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B436" s="0" t="n">
+        <v>852</v>
+      </c>
+      <c r="C436" s="0" t="n">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B437" s="0" t="n">
+        <v>974</v>
+      </c>
+      <c r="C437" s="0" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B438" s="0" t="n">
+        <v>738</v>
+      </c>
+      <c r="C438" s="0" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B439" s="0" t="n">
+        <v>521</v>
+      </c>
+      <c r="C439" s="0" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B440" s="0" t="n">
+        <v>943</v>
+      </c>
+      <c r="C440" s="0" t="n">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B441" s="0" t="n">
+        <v>92</v>
+      </c>
+      <c r="C441" s="0" t="n">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B442" s="0" t="n">
+        <v>268</v>
+      </c>
+      <c r="C442" s="0" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B443" s="0" t="n">
+        <v>792</v>
+      </c>
+      <c r="C443" s="0" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B444" s="0" t="n">
+        <v>344</v>
+      </c>
+      <c r="C444" s="0" t="n">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B445" s="0" t="n">
+        <v>941</v>
+      </c>
+      <c r="C445" s="0" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B446" s="0" t="n">
+        <v>1190</v>
+      </c>
+      <c r="C446" s="0" t="n">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B447" s="0" t="n">
+        <v>1147</v>
+      </c>
+      <c r="C447" s="0" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B448" s="0" t="n">
+        <v>91</v>
+      </c>
+      <c r="C448" s="0" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B449" s="0" t="n">
+        <v>822</v>
+      </c>
+      <c r="C449" s="0" t="n">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B450" s="0" t="n">
+        <v>664</v>
+      </c>
+      <c r="C450" s="0" t="n">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B451" s="0" t="n">
+        <v>791</v>
+      </c>
+      <c r="C451" s="0" t="n">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B452" s="0" t="n">
+        <v>1077</v>
+      </c>
+      <c r="C452" s="0" t="n">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B453" s="0" t="n">
+        <v>431</v>
+      </c>
+      <c r="C453" s="0" t="n">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B454" s="0" t="n">
+        <v>147</v>
+      </c>
+      <c r="C454" s="0" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B455" s="0" t="n">
+        <v>778</v>
+      </c>
+      <c r="C455" s="0" t="n">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B456" s="0" t="n">
+        <v>1040</v>
+      </c>
+      <c r="C456" s="0" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B457" s="0" t="n">
+        <v>105</v>
+      </c>
+      <c r="C457" s="0" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B458" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C458" s="0" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B459" s="0" t="n">
+        <v>950</v>
+      </c>
+      <c r="C459" s="0" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B460" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C460" s="0" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B461" s="0" t="n">
+        <v>707</v>
+      </c>
+      <c r="C461" s="0" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B462" s="0" t="n">
+        <v>909</v>
+      </c>
+      <c r="C462" s="0" t="n">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B463" s="0" t="n">
+        <v>736</v>
+      </c>
+      <c r="C463" s="0" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B464" s="0" t="n">
+        <v>1107</v>
+      </c>
+      <c r="C464" s="0" t="n">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B465" s="0" t="n">
+        <v>1141</v>
+      </c>
+      <c r="C465" s="0" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B466" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C466" s="0" t="n">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B467" s="0" t="n">
+        <v>347</v>
+      </c>
+      <c r="C467" s="0" t="n">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B468" s="0" t="n">
+        <v>201</v>
+      </c>
+      <c r="C468" s="0" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B469" s="0" t="n">
+        <v>923</v>
+      </c>
+      <c r="C469" s="0" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B470" s="0" t="n">
+        <v>1198</v>
+      </c>
+      <c r="C470" s="0" t="n">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B471" s="0" t="n">
+        <v>743</v>
+      </c>
+      <c r="C471" s="0" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B472" s="0" t="n">
+        <v>720</v>
+      </c>
+      <c r="C472" s="0" t="n">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B473" s="0" t="n">
+        <v>199</v>
+      </c>
+      <c r="C473" s="0" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B474" s="0" t="n">
+        <v>716</v>
+      </c>
+      <c r="C474" s="0" t="n">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B475" s="0" t="n">
+        <v>802</v>
+      </c>
+      <c r="C475" s="0" t="n">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B476" s="0" t="n">
+        <v>391</v>
+      </c>
+      <c r="C476" s="0" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B477" s="0" t="n">
+        <v>902</v>
+      </c>
+      <c r="C477" s="0" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B478" s="0" t="n">
+        <v>135</v>
+      </c>
+      <c r="C478" s="0" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B479" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C479" s="0" t="n">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B480" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="C480" s="0" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B481" s="0" t="n">
+        <v>92</v>
+      </c>
+      <c r="C481" s="0" t="n">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B482" s="0" t="n">
+        <v>382</v>
+      </c>
+      <c r="C482" s="0" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B483" s="0" t="n">
+        <v>675</v>
+      </c>
+      <c r="C483" s="0" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B484" s="0" t="n">
+        <v>983</v>
+      </c>
+      <c r="C484" s="0" t="n">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B485" s="0" t="n">
+        <v>1087</v>
+      </c>
+      <c r="C485" s="0" t="n">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B486" s="0" t="n">
+        <v>278</v>
+      </c>
+      <c r="C486" s="0" t="n">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B487" s="0" t="n">
+        <v>1090</v>
+      </c>
+      <c r="C487" s="0" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B488" s="0" t="n">
+        <v>667</v>
+      </c>
+      <c r="C488" s="0" t="n">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B489" s="0" t="n">
+        <v>734</v>
+      </c>
+      <c r="C489" s="0" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B490" s="0" t="n">
+        <v>270</v>
+      </c>
+      <c r="C490" s="0" t="n">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B491" s="0" t="n">
+        <v>907</v>
+      </c>
+      <c r="C491" s="0" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B492" s="0" t="n">
+        <v>1185</v>
+      </c>
+      <c r="C492" s="0" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B493" s="0" t="n">
+        <v>978</v>
+      </c>
+      <c r="C493" s="0" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B494" s="0" t="n">
+        <v>846</v>
+      </c>
+      <c r="C494" s="0" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B495" s="0" t="n">
+        <v>386</v>
+      </c>
+      <c r="C495" s="0" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B496" s="0" t="n">
+        <v>510</v>
+      </c>
+      <c r="C496" s="0" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B497" s="0" t="n">
+        <v>1067</v>
+      </c>
+      <c r="C497" s="0" t="n">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B498" s="0" t="n">
+        <v>184</v>
+      </c>
+      <c r="C498" s="0" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B499" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C499" s="0" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B500" s="0" t="n">
+        <v>998</v>
+      </c>
+      <c r="C500" s="0" t="n">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B501" s="0" t="n">
+        <v>468</v>
+      </c>
+      <c r="C501" s="0" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="B502" s="0" t="n">
+        <v>889</v>
+      </c>
+      <c r="C502" s="0" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="B503" s="0" t="n">
+        <v>618</v>
+      </c>
+      <c r="C503" s="0" t="n">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="0" t="n">
+        <v>53</v>
+      </c>
+      <c r="B504" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C504" s="0" t="n">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="0" t="n">
+        <v>54</v>
+      </c>
+      <c r="B505" s="0" t="n">
+        <v>392</v>
+      </c>
+      <c r="C505" s="0" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="B506" s="0" t="n">
+        <v>274</v>
+      </c>
+      <c r="C506" s="0" t="n">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="0" t="n">
+        <v>56</v>
+      </c>
+      <c r="B507" s="0" t="n">
+        <v>228</v>
+      </c>
+      <c r="C507" s="0" t="n">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="0" t="n">
+        <v>57</v>
+      </c>
+      <c r="B508" s="0" t="n">
+        <v>948</v>
+      </c>
+      <c r="C508" s="0" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="0" t="n">
+        <v>58</v>
+      </c>
+      <c r="B509" s="0" t="n">
+        <v>792</v>
+      </c>
+      <c r="C509" s="0" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="0" t="n">
+        <v>59</v>
+      </c>
+      <c r="B510" s="0" t="n">
+        <v>1113</v>
+      </c>
+      <c r="C510" s="0" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="B511" s="0" t="n">
+        <v>967</v>
+      </c>
+      <c r="C511" s="0" t="n">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="0" t="n">
+        <v>61</v>
+      </c>
+      <c r="B512" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C512" s="0" t="n">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="0" t="n">
+        <v>62</v>
+      </c>
+      <c r="B513" s="0" t="n">
+        <v>906</v>
+      </c>
+      <c r="C513" s="0" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="0" t="n">
+        <v>63</v>
+      </c>
+      <c r="B514" s="0" t="n">
+        <v>767</v>
+      </c>
+      <c r="C514" s="0" t="n">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="0" t="n">
+        <v>64</v>
+      </c>
+      <c r="B515" s="0" t="n">
+        <v>294</v>
+      </c>
+      <c r="C515" s="0" t="n">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="0" t="n">
+        <v>65</v>
+      </c>
+      <c r="B516" s="0" t="n">
+        <v>109</v>
+      </c>
+      <c r="C516" s="0" t="n">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="B517" s="0" t="n">
+        <v>531</v>
+      </c>
+      <c r="C517" s="0" t="n">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="0" t="n">
+        <v>67</v>
+      </c>
+      <c r="B518" s="0" t="n">
+        <v>638</v>
+      </c>
+      <c r="C518" s="0" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="0" t="n">
+        <v>68</v>
+      </c>
+      <c r="B519" s="0" t="n">
+        <v>767</v>
+      </c>
+      <c r="C519" s="0" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="0" t="n">
+        <v>69</v>
+      </c>
+      <c r="B520" s="0" t="n">
+        <v>708</v>
+      </c>
+      <c r="C520" s="0" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="0" t="n">
+        <v>70</v>
+      </c>
+      <c r="B521" s="0" t="n">
+        <v>769</v>
+      </c>
+      <c r="C521" s="0" t="n">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="B522" s="0" t="n">
+        <v>956</v>
+      </c>
+      <c r="C522" s="0" t="n">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="0" t="n">
+        <v>72</v>
+      </c>
+      <c r="B523" s="0" t="n">
+        <v>86</v>
+      </c>
+      <c r="C523" s="0" t="n">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="B524" s="0" t="n">
+        <v>1048</v>
+      </c>
+      <c r="C524" s="0" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="0" t="n">
+        <v>74</v>
+      </c>
+      <c r="B525" s="0" t="n">
+        <v>650</v>
+      </c>
+      <c r="C525" s="0" t="n">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="B526" s="0" t="n">
+        <v>263</v>
+      </c>
+      <c r="C526" s="0" t="n">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="0" t="n">
+        <v>76</v>
+      </c>
+      <c r="B527" s="0" t="n">
+        <v>1170</v>
+      </c>
+      <c r="C527" s="0" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="0" t="n">
+        <v>77</v>
+      </c>
+      <c r="B528" s="0" t="n">
+        <v>782</v>
+      </c>
+      <c r="C528" s="0" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="0" t="n">
+        <v>78</v>
+      </c>
+      <c r="B529" s="0" t="n">
+        <v>215</v>
+      </c>
+      <c r="C529" s="0" t="n">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="0" t="n">
+        <v>79</v>
+      </c>
+      <c r="B530" s="0" t="n">
+        <v>660</v>
+      </c>
+      <c r="C530" s="0" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="0" t="n">
+        <v>80</v>
+      </c>
+      <c r="B531" s="0" t="n">
+        <v>892</v>
+      </c>
+      <c r="C531" s="0" t="n">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="0" t="n">
+        <v>81</v>
+      </c>
+      <c r="B532" s="0" t="n">
+        <v>1057</v>
+      </c>
+      <c r="C532" s="0" t="n">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="0" t="n">
+        <v>82</v>
+      </c>
+      <c r="B533" s="0" t="n">
+        <v>1052</v>
+      </c>
+      <c r="C533" s="0" t="n">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="0" t="n">
+        <v>83</v>
+      </c>
+      <c r="B534" s="0" t="n">
+        <v>593</v>
+      </c>
+      <c r="C534" s="0" t="n">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="0" t="n">
+        <v>84</v>
+      </c>
+      <c r="B535" s="0" t="n">
+        <v>611</v>
+      </c>
+      <c r="C535" s="0" t="n">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="0" t="n">
+        <v>85</v>
+      </c>
+      <c r="B536" s="0" t="n">
+        <v>452</v>
+      </c>
+      <c r="C536" s="0" t="n">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="0" t="n">
+        <v>86</v>
+      </c>
+      <c r="B537" s="0" t="n">
+        <v>703</v>
+      </c>
+      <c r="C537" s="0" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="0" t="n">
+        <v>87</v>
+      </c>
+      <c r="B538" s="0" t="n">
+        <v>724</v>
+      </c>
+      <c r="C538" s="0" t="n">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="0" t="n">
+        <v>88</v>
+      </c>
+      <c r="B539" s="0" t="n">
+        <v>1017</v>
+      </c>
+      <c r="C539" s="0" t="n">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="0" t="n">
+        <v>89</v>
+      </c>
+      <c r="B540" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="C540" s="0" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="B541" s="0" t="n">
+        <v>1155</v>
+      </c>
+      <c r="C541" s="0" t="n">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="0" t="n">
+        <v>91</v>
+      </c>
+      <c r="B542" s="0" t="n">
+        <v>283</v>
+      </c>
+      <c r="C542" s="0" t="n">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="0" t="n">
+        <v>92</v>
+      </c>
+      <c r="B543" s="0" t="n">
+        <v>1156</v>
+      </c>
+      <c r="C543" s="0" t="n">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="0" t="n">
+        <v>93</v>
+      </c>
+      <c r="B544" s="0" t="n">
+        <v>985</v>
+      </c>
+      <c r="C544" s="0" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="0" t="n">
+        <v>94</v>
+      </c>
+      <c r="B545" s="0" t="n">
+        <v>661</v>
+      </c>
+      <c r="C545" s="0" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="0" t="n">
+        <v>95</v>
+      </c>
+      <c r="B546" s="0" t="n">
+        <v>383</v>
+      </c>
+      <c r="C546" s="0" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="0" t="n">
+        <v>96</v>
+      </c>
+      <c r="B547" s="0" t="n">
+        <v>336</v>
+      </c>
+      <c r="C547" s="0" t="n">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="0" t="n">
+        <v>97</v>
+      </c>
+      <c r="B548" s="0" t="n">
+        <v>569</v>
+      </c>
+      <c r="C548" s="0" t="n">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="0" t="n">
+        <v>98</v>
+      </c>
+      <c r="B549" s="0" t="n">
+        <v>1051</v>
+      </c>
+      <c r="C549" s="0" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="B550" s="0" t="n">
+        <v>1040</v>
+      </c>
+      <c r="C550" s="0" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="B551" s="0" t="n">
+        <v>782</v>
+      </c>
+      <c r="C551" s="0" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B552" s="0" t="n">
+        <v>70</v>
+      </c>
+      <c r="C552" s="0" t="n">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B553" s="0" t="n">
+        <v>631</v>
+      </c>
+      <c r="C553" s="0" t="n">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B554" s="0" t="n">
+        <v>381</v>
+      </c>
+      <c r="C554" s="0" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B555" s="0" t="n">
+        <v>573</v>
+      </c>
+      <c r="C555" s="0" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B556" s="0" t="n">
+        <v>412</v>
+      </c>
+      <c r="C556" s="0" t="n">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B557" s="0" t="n">
+        <v>913</v>
+      </c>
+      <c r="C557" s="0" t="n">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B558" s="0" t="n">
+        <v>498</v>
+      </c>
+      <c r="C558" s="0" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B559" s="0" t="n">
+        <v>942</v>
+      </c>
+      <c r="C559" s="0" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B560" s="0" t="n">
+        <v>368</v>
+      </c>
+      <c r="C560" s="0" t="n">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B561" s="0" t="n">
+        <v>217</v>
+      </c>
+      <c r="C561" s="0" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B562" s="0" t="n">
+        <v>454</v>
+      </c>
+      <c r="C562" s="0" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B563" s="0" t="n">
+        <v>248</v>
+      </c>
+      <c r="C563" s="0" t="n">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B564" s="0" t="n">
+        <v>463</v>
+      </c>
+      <c r="C564" s="0" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B565" s="0" t="n">
+        <v>187</v>
+      </c>
+      <c r="C565" s="0" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B566" s="0" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C566" s="0" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B567" s="0" t="n">
+        <v>193</v>
+      </c>
+      <c r="C567" s="0" t="n">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B568" s="0" t="n">
+        <v>339</v>
+      </c>
+      <c r="C568" s="0" t="n">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B569" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C569" s="0" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B570" s="0" t="n">
+        <v>63</v>
+      </c>
+      <c r="C570" s="0" t="n">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B571" s="0" t="n">
+        <v>700</v>
+      </c>
+      <c r="C571" s="0" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B572" s="0" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C572" s="0" t="n">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B573" s="0" t="n">
+        <v>793</v>
+      </c>
+      <c r="C573" s="0" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B574" s="0" t="n">
+        <v>690</v>
+      </c>
+      <c r="C574" s="0" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B575" s="0" t="n">
+        <v>775</v>
+      </c>
+      <c r="C575" s="0" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B576" s="0" t="n">
+        <v>190</v>
+      </c>
+      <c r="C576" s="0" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B577" s="0" t="n">
+        <v>1174</v>
+      </c>
+      <c r="C577" s="0" t="n">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B578" s="0" t="n">
+        <v>1183</v>
+      </c>
+      <c r="C578" s="0" t="n">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B579" s="0" t="n">
+        <v>1082</v>
+      </c>
+      <c r="C579" s="0" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B580" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C580" s="0" t="n">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B581" s="0" t="n">
+        <v>535</v>
+      </c>
+      <c r="C581" s="0" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B582" s="0" t="n">
+        <v>61</v>
+      </c>
+      <c r="C582" s="0" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B583" s="0" t="n">
+        <v>335</v>
+      </c>
+      <c r="C583" s="0" t="n">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B584" s="0" t="n">
+        <v>1133</v>
+      </c>
+      <c r="C584" s="0" t="n">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B585" s="0" t="n">
+        <v>798</v>
+      </c>
+      <c r="C585" s="0" t="n">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B586" s="0" t="n">
+        <v>646</v>
+      </c>
+      <c r="C586" s="0" t="n">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B587" s="0" t="n">
+        <v>477</v>
+      </c>
+      <c r="C587" s="0" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B588" s="0" t="n">
+        <v>179</v>
+      </c>
+      <c r="C588" s="0" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B589" s="0" t="n">
+        <v>1194</v>
+      </c>
+      <c r="C589" s="0" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B590" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="C590" s="0" t="n">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B591" s="0" t="n">
+        <v>810</v>
+      </c>
+      <c r="C591" s="0" t="n">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B592" s="0" t="n">
+        <v>1194</v>
+      </c>
+      <c r="C592" s="0" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B593" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="C593" s="0" t="n">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B594" s="0" t="n">
+        <v>945</v>
+      </c>
+      <c r="C594" s="0" t="n">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B595" s="0" t="n">
+        <v>1054</v>
+      </c>
+      <c r="C595" s="0" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B596" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C596" s="0" t="n">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B597" s="0" t="n">
+        <v>858</v>
+      </c>
+      <c r="C597" s="0" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B598" s="0" t="n">
+        <v>570</v>
+      </c>
+      <c r="C598" s="0" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B599" s="0" t="n">
+        <v>460</v>
+      </c>
+      <c r="C599" s="0" t="n">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B600" s="0" t="n">
+        <v>194</v>
+      </c>
+      <c r="C600" s="0" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B601" s="0" t="n">
+        <v>889</v>
+      </c>
+      <c r="C601" s="0" t="n">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B602" s="0" t="n">
+        <v>57</v>
+      </c>
+      <c r="C602" s="0" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B603" s="0" t="n">
+        <v>654</v>
+      </c>
+      <c r="C603" s="0" t="n">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B604" s="0" t="n">
+        <v>591</v>
+      </c>
+      <c r="C604" s="0" t="n">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B605" s="0" t="n">
+        <v>747</v>
+      </c>
+      <c r="C605" s="0" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B606" s="0" t="n">
+        <v>102</v>
+      </c>
+      <c r="C606" s="0" t="n">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B607" s="0" t="n">
+        <v>448</v>
+      </c>
+      <c r="C607" s="0" t="n">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B608" s="0" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C608" s="0" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B609" s="0" t="n">
+        <v>258</v>
+      </c>
+      <c r="C609" s="0" t="n">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B610" s="0" t="n">
+        <v>785</v>
+      </c>
+      <c r="C610" s="0" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B611" s="0" t="n">
+        <v>62</v>
+      </c>
+      <c r="C611" s="0" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B612" s="0" t="n">
+        <v>884</v>
+      </c>
+      <c r="C612" s="0" t="n">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B613" s="0" t="n">
+        <v>1156</v>
+      </c>
+      <c r="C613" s="0" t="n">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B614" s="0" t="n">
+        <v>328</v>
+      </c>
+      <c r="C614" s="0" t="n">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B615" s="0" t="n">
+        <v>998</v>
+      </c>
+      <c r="C615" s="0" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B616" s="0" t="n">
+        <v>373</v>
+      </c>
+      <c r="C616" s="0" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B617" s="0" t="n">
+        <v>879</v>
+      </c>
+      <c r="C617" s="0" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B618" s="0" t="n">
+        <v>398</v>
+      </c>
+      <c r="C618" s="0" t="n">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B619" s="0" t="n">
+        <v>854</v>
+      </c>
+      <c r="C619" s="0" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B620" s="0" t="n">
+        <v>457</v>
+      </c>
+      <c r="C620" s="0" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B621" s="0" t="n">
+        <v>499</v>
+      </c>
+      <c r="C621" s="0" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="B622" s="0" t="n">
+        <v>552</v>
+      </c>
+      <c r="C622" s="0" t="n">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="B623" s="0" t="n">
+        <v>170</v>
+      </c>
+      <c r="C623" s="0" t="n">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B624" s="0" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C624" s="0" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B625" s="0" t="n">
+        <v>1130</v>
+      </c>
+      <c r="C625" s="0" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B626" s="0" t="n">
+        <v>842</v>
+      </c>
+      <c r="C626" s="0" t="n">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B627" s="0" t="n">
+        <v>385</v>
+      </c>
+      <c r="C627" s="0" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B628" s="0" t="n">
+        <v>932</v>
+      </c>
+      <c r="C628" s="0" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B629" s="0" t="n">
+        <v>531</v>
+      </c>
+      <c r="C629" s="0" t="n">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B630" s="0" t="n">
+        <v>849</v>
+      </c>
+      <c r="C630" s="0" t="n">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B631" s="0" t="n">
+        <v>1158</v>
+      </c>
+      <c r="C631" s="0" t="n">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B632" s="0" t="n">
+        <v>688</v>
+      </c>
+      <c r="C632" s="0" t="n">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B633" s="0" t="n">
+        <v>561</v>
+      </c>
+      <c r="C633" s="0" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B634" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C634" s="0" t="n">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B635" s="0" t="n">
+        <v>956</v>
+      </c>
+      <c r="C635" s="0" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B636" s="0" t="n">
+        <v>868</v>
+      </c>
+      <c r="C636" s="0" t="n">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B637" s="0" t="n">
+        <v>1085</v>
+      </c>
+      <c r="C637" s="0" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B638" s="0" t="n">
+        <v>994</v>
+      </c>
+      <c r="C638" s="0" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B639" s="0" t="n">
+        <v>596</v>
+      </c>
+      <c r="C639" s="0" t="n">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B640" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C640" s="0" t="n">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B641" s="0" t="n">
+        <v>562</v>
+      </c>
+      <c r="C641" s="0" t="n">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B642" s="0" t="n">
+        <v>854</v>
+      </c>
+      <c r="C642" s="0" t="n">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B643" s="0" t="n">
+        <v>672</v>
+      </c>
+      <c r="C643" s="0" t="n">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B644" s="0" t="n">
+        <v>909</v>
+      </c>
+      <c r="C644" s="0" t="n">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B645" s="0" t="n">
+        <v>1065</v>
+      </c>
+      <c r="C645" s="0" t="n">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B646" s="0" t="n">
+        <v>638</v>
+      </c>
+      <c r="C646" s="0" t="n">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B647" s="0" t="n">
+        <v>488</v>
+      </c>
+      <c r="C647" s="0" t="n">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B648" s="0" t="n">
+        <v>908</v>
+      </c>
+      <c r="C648" s="0" t="n">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B649" s="0" t="n">
+        <v>918</v>
+      </c>
+      <c r="C649" s="0" t="n">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B650" s="0" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C650" s="0" t="n">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B651" s="0" t="n">
+        <v>660</v>
+      </c>
+      <c r="C651" s="0" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B652" s="0" t="n">
+        <v>976</v>
+      </c>
+      <c r="C652" s="0" t="n">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B653" s="0" t="n">
+        <v>249</v>
+      </c>
+      <c r="C653" s="0" t="n">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B654" s="0" t="n">
+        <v>990</v>
+      </c>
+      <c r="C654" s="0" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B655" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C655" s="0" t="n">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B656" s="0" t="n">
+        <v>301</v>
+      </c>
+      <c r="C656" s="0" t="n">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B657" s="0" t="n">
+        <v>734</v>
+      </c>
+      <c r="C657" s="0" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B658" s="0" t="n">
+        <v>134</v>
+      </c>
+      <c r="C658" s="0" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B659" s="0" t="n">
+        <v>695</v>
+      </c>
+      <c r="C659" s="0" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B660" s="0" t="n">
+        <v>662</v>
+      </c>
+      <c r="C660" s="0" t="n">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B661" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="C661" s="0" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B662" s="0" t="n">
+        <v>976</v>
+      </c>
+      <c r="C662" s="0" t="n">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B663" s="0" t="n">
+        <v>431</v>
+      </c>
+      <c r="C663" s="0" t="n">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B664" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C664" s="0" t="n">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B665" s="0" t="n">
+        <v>603</v>
+      </c>
+      <c r="C665" s="0" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B666" s="0" t="n">
+        <v>1158</v>
+      </c>
+      <c r="C666" s="0" t="n">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B667" s="0" t="n">
+        <v>796</v>
+      </c>
+      <c r="C667" s="0" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B668" s="0" t="n">
+        <v>295</v>
+      </c>
+      <c r="C668" s="0" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B669" s="0" t="n">
+        <v>211</v>
+      </c>
+      <c r="C669" s="0" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B670" s="0" t="n">
+        <v>312</v>
+      </c>
+      <c r="C670" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B671" s="0" t="n">
+        <v>618</v>
+      </c>
+      <c r="C671" s="0" t="n">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B672" s="0" t="n">
+        <v>1151</v>
+      </c>
+      <c r="C672" s="0" t="n">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B673" s="0" t="n">
+        <v>424</v>
+      </c>
+      <c r="C673" s="0" t="n">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B674" s="0" t="n">
+        <v>895</v>
+      </c>
+      <c r="C674" s="0" t="n">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B675" s="0" t="n">
+        <v>831</v>
+      </c>
+      <c r="C675" s="0" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B676" s="0" t="n">
+        <v>665</v>
+      </c>
+      <c r="C676" s="0" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B677" s="0" t="n">
+        <v>687</v>
+      </c>
+      <c r="C677" s="0" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B678" s="0" t="n">
+        <v>719</v>
+      </c>
+      <c r="C678" s="0" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B679" s="0" t="n">
+        <v>87</v>
+      </c>
+      <c r="C679" s="0" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B680" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C680" s="0" t="n">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B681" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="C681" s="0" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B682" s="0" t="n">
+        <v>703</v>
+      </c>
+      <c r="C682" s="0" t="n">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B683" s="0" t="n">
+        <v>788</v>
+      </c>
+      <c r="C683" s="0" t="n">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B684" s="0" t="n">
+        <v>895</v>
+      </c>
+      <c r="C684" s="0" t="n">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B685" s="0" t="n">
+        <v>846</v>
+      </c>
+      <c r="C685" s="0" t="n">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B686" s="0" t="n">
+        <v>273</v>
+      </c>
+      <c r="C686" s="0" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B687" s="0" t="n">
+        <v>609</v>
+      </c>
+      <c r="C687" s="0" t="n">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B688" s="0" t="n">
+        <v>747</v>
+      </c>
+      <c r="C688" s="0" t="n">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B689" s="0" t="n">
+        <v>439</v>
+      </c>
+      <c r="C689" s="0" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B690" s="0" t="n">
+        <v>804</v>
+      </c>
+      <c r="C690" s="0" t="n">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B691" s="0" t="n">
+        <v>72</v>
+      </c>
+      <c r="C691" s="0" t="n">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B692" s="0" t="n">
+        <v>205</v>
+      </c>
+      <c r="C692" s="0" t="n">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B693" s="0" t="n">
+        <v>537</v>
+      </c>
+      <c r="C693" s="0" t="n">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B694" s="0" t="n">
+        <v>627</v>
+      </c>
+      <c r="C694" s="0" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B695" s="0" t="n">
+        <v>433</v>
+      </c>
+      <c r="C695" s="0" t="n">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B696" s="0" t="n">
+        <v>740</v>
+      </c>
+      <c r="C696" s="0" t="n">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B697" s="0" t="n">
+        <v>442</v>
+      </c>
+      <c r="C697" s="0" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B698" s="0" t="n">
+        <v>348</v>
+      </c>
+      <c r="C698" s="0" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B699" s="0" t="n">
+        <v>1131</v>
+      </c>
+      <c r="C699" s="0" t="n">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B700" s="0" t="n">
+        <v>686</v>
+      </c>
+      <c r="C700" s="0" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B701" s="0" t="n">
+        <v>860</v>
+      </c>
+      <c r="C701" s="0" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B702" s="0" t="n">
+        <v>843</v>
+      </c>
+      <c r="C702" s="0" t="n">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B703" s="0" t="n">
+        <v>954</v>
+      </c>
+      <c r="C703" s="0" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B704" s="0" t="n">
+        <v>476</v>
+      </c>
+      <c r="C704" s="0" t="n">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B705" s="0" t="n">
+        <v>904</v>
+      </c>
+      <c r="C705" s="0" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B706" s="0" t="n">
+        <v>327</v>
+      </c>
+      <c r="C706" s="0" t="n">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B707" s="0" t="n">
+        <v>861</v>
+      </c>
+      <c r="C707" s="0" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B708" s="0" t="n">
+        <v>634</v>
+      </c>
+      <c r="C708" s="0" t="n">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B709" s="0" t="n">
+        <v>1053</v>
+      </c>
+      <c r="C709" s="0" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B710" s="0" t="n">
+        <v>282</v>
+      </c>
+      <c r="C710" s="0" t="n">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B711" s="0" t="n">
+        <v>991</v>
+      </c>
+      <c r="C711" s="0" t="n">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B712" s="0" t="n">
+        <v>425</v>
+      </c>
+      <c r="C712" s="0" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B713" s="0" t="n">
+        <v>110</v>
+      </c>
+      <c r="C713" s="0" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B714" s="0" t="n">
+        <v>619</v>
+      </c>
+      <c r="C714" s="0" t="n">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B715" s="0" t="n">
+        <v>424</v>
+      </c>
+      <c r="C715" s="0" t="n">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B716" s="0" t="n">
+        <v>147</v>
+      </c>
+      <c r="C716" s="0" t="n">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B717" s="0" t="n">
+        <v>772</v>
+      </c>
+      <c r="C717" s="0" t="n">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B718" s="0" t="n">
+        <v>910</v>
+      </c>
+      <c r="C718" s="0" t="n">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B719" s="0" t="n">
+        <v>536</v>
+      </c>
+      <c r="C719" s="0" t="n">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B720" s="0" t="n">
+        <v>485</v>
+      </c>
+      <c r="C720" s="0" t="n">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B721" s="0" t="n">
+        <v>600</v>
+      </c>
+      <c r="C721" s="0" t="n">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B722" s="0" t="n">
+        <v>662</v>
+      </c>
+      <c r="C722" s="0" t="n">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B723" s="0" t="n">
+        <v>1017</v>
+      </c>
+      <c r="C723" s="0" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B724" s="0" t="n">
+        <v>884</v>
+      </c>
+      <c r="C724" s="0" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B725" s="0" t="n">
+        <v>312</v>
+      </c>
+      <c r="C725" s="0" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B726" s="0" t="n">
+        <v>1199</v>
+      </c>
+      <c r="C726" s="0" t="n">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B727" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C727" s="0" t="n">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B728" s="0" t="n">
+        <v>378</v>
+      </c>
+      <c r="C728" s="0" t="n">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B729" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C729" s="0" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B730" s="0" t="n">
+        <v>562</v>
+      </c>
+      <c r="C730" s="0" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B731" s="0" t="n">
+        <v>177</v>
+      </c>
+      <c r="C731" s="0" t="n">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B732" s="0" t="n">
+        <v>592</v>
+      </c>
+      <c r="C732" s="0" t="n">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B733" s="0" t="n">
+        <v>674</v>
+      </c>
+      <c r="C733" s="0" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B734" s="0" t="n">
+        <v>920</v>
+      </c>
+      <c r="C734" s="0" t="n">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B735" s="0" t="n">
+        <v>1108</v>
+      </c>
+      <c r="C735" s="0" t="n">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B736" s="0" t="n">
+        <v>1079</v>
+      </c>
+      <c r="C736" s="0" t="n">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B737" s="0" t="n">
+        <v>454</v>
+      </c>
+      <c r="C737" s="0" t="n">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B738" s="0" t="n">
+        <v>193</v>
+      </c>
+      <c r="C738" s="0" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B739" s="0" t="n">
+        <v>1197</v>
+      </c>
+      <c r="C739" s="0" t="n">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B740" s="0" t="n">
+        <v>710</v>
+      </c>
+      <c r="C740" s="0" t="n">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B741" s="0" t="n">
+        <v>955</v>
+      </c>
+      <c r="C741" s="0" t="n">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B742" s="0" t="n">
+        <v>80</v>
+      </c>
+      <c r="C742" s="0" t="n">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B743" s="0" t="n">
+        <v>1103</v>
+      </c>
+      <c r="C743" s="0" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="n">
+        <v>1</v>
+      </c>
+      <c r="B744" t="n">
+        <v>176</v>
+      </c>
+      <c r="C744" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="n">
+        <v>2</v>
+      </c>
+      <c r="B745" t="n">
+        <v>24</v>
+      </c>
+      <c r="C745" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="n">
+        <v>3</v>
+      </c>
+      <c r="B746" t="n">
+        <v>59</v>
+      </c>
+      <c r="C746" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="n">
+        <v>4</v>
+      </c>
+      <c r="B747" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C747" t="n">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="n">
+        <v>5</v>
+      </c>
+      <c r="B748" t="n">
+        <v>779</v>
+      </c>
+      <c r="C748" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="n">
+        <v>6</v>
+      </c>
+      <c r="B749" t="n">
+        <v>184</v>
+      </c>
+      <c r="C749" t="n">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="n">
+        <v>7</v>
+      </c>
+      <c r="B750" t="n">
+        <v>976</v>
+      </c>
+      <c r="C750" t="n">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>8</v>
+      </c>
+      <c r="B751" t="n">
+        <v>496</v>
+      </c>
+      <c r="C751" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>9</v>
+      </c>
+      <c r="B752" t="n">
+        <v>757</v>
+      </c>
+      <c r="C752" t="n">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="n">
+        <v>10</v>
+      </c>
+      <c r="B753" t="n">
+        <v>561</v>
+      </c>
+      <c r="C753" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>11</v>
+      </c>
+      <c r="B754" t="n">
+        <v>788</v>
+      </c>
+      <c r="C754" t="n">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>12</v>
+      </c>
+      <c r="B755" t="n">
+        <v>672</v>
+      </c>
+      <c r="C755" t="n">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="n">
+        <v>13</v>
+      </c>
+      <c r="B756" t="n">
+        <v>441</v>
+      </c>
+      <c r="C756" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="n">
+        <v>14</v>
+      </c>
+      <c r="B757" t="n">
+        <v>1072</v>
+      </c>
+      <c r="C757" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="n">
+        <v>15</v>
+      </c>
+      <c r="B758" t="n">
+        <v>857</v>
+      </c>
+      <c r="C758" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="n">
+        <v>16</v>
+      </c>
+      <c r="B759" t="n">
+        <v>654</v>
+      </c>
+      <c r="C759" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="n">
+        <v>17</v>
+      </c>
+      <c r="B760" t="n">
+        <v>447</v>
+      </c>
+      <c r="C760" t="n">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="n">
+        <v>18</v>
+      </c>
+      <c r="B761" t="n">
+        <v>1052</v>
+      </c>
+      <c r="C761" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="n">
+        <v>19</v>
+      </c>
+      <c r="B762" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C762" t="n">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="n">
+        <v>20</v>
+      </c>
+      <c r="B763" t="n">
+        <v>207</v>
+      </c>
+      <c r="C763" t="n">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="n">
+        <v>21</v>
+      </c>
+      <c r="B764" t="n">
+        <v>525</v>
+      </c>
+      <c r="C764" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="n">
+        <v>22</v>
+      </c>
+      <c r="B765" t="n">
+        <v>585</v>
+      </c>
+      <c r="C765" t="n">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="n">
+        <v>23</v>
+      </c>
+      <c r="B766" t="n">
+        <v>939</v>
+      </c>
+      <c r="C766" t="n">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="n">
+        <v>24</v>
+      </c>
+      <c r="B767" t="n">
+        <v>714</v>
+      </c>
+      <c r="C767" t="n">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="n">
+        <v>25</v>
+      </c>
+      <c r="B768" t="n">
+        <v>305</v>
+      </c>
+      <c r="C768" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="n">
+        <v>26</v>
+      </c>
+      <c r="B769" t="n">
+        <v>909</v>
+      </c>
+      <c r="C769" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="n">
+        <v>27</v>
+      </c>
+      <c r="B770" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C770" t="n">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="n">
+        <v>28</v>
+      </c>
+      <c r="B771" t="n">
+        <v>937</v>
+      </c>
+      <c r="C771" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="n">
+        <v>29</v>
+      </c>
+      <c r="B772" t="n">
+        <v>747</v>
+      </c>
+      <c r="C772" t="n">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="n">
+        <v>30</v>
+      </c>
+      <c r="B773" t="n">
+        <v>188</v>
+      </c>
+      <c r="C773" t="n">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="n">
+        <v>31</v>
+      </c>
+      <c r="B774" t="n">
+        <v>17</v>
+      </c>
+      <c r="C774" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="n">
+        <v>32</v>
+      </c>
+      <c r="B775" t="n">
+        <v>747</v>
+      </c>
+      <c r="C775" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="n">
+        <v>33</v>
+      </c>
+      <c r="B776" t="n">
+        <v>460</v>
+      </c>
+      <c r="C776" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="n">
+        <v>34</v>
+      </c>
+      <c r="B777" t="n">
+        <v>315</v>
+      </c>
+      <c r="C777" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="n">
+        <v>35</v>
+      </c>
+      <c r="B778" t="n">
+        <v>393</v>
+      </c>
+      <c r="C778" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="n">
+        <v>36</v>
+      </c>
+      <c r="B779" t="n">
+        <v>832</v>
+      </c>
+      <c r="C779" t="n">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="n">
+        <v>37</v>
+      </c>
+      <c r="B780" t="n">
+        <v>765</v>
+      </c>
+      <c r="C780" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>38</v>
+      </c>
+      <c r="B781" t="n">
+        <v>1055</v>
+      </c>
+      <c r="C781" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="n">
+        <v>39</v>
+      </c>
+      <c r="B782" t="n">
+        <v>200</v>
+      </c>
+      <c r="C782" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="n">
+        <v>40</v>
+      </c>
+      <c r="B783" t="n">
+        <v>549</v>
+      </c>
+      <c r="C783" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="n">
+        <v>41</v>
+      </c>
+      <c r="B784" t="n">
+        <v>115</v>
+      </c>
+      <c r="C784" t="n">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="n">
+        <v>42</v>
+      </c>
+      <c r="B785" t="n">
+        <v>880</v>
+      </c>
+      <c r="C785" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="n">
+        <v>43</v>
+      </c>
+      <c r="B786" t="n">
+        <v>918</v>
+      </c>
+      <c r="C786" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="n">
+        <v>44</v>
+      </c>
+      <c r="B787" t="n">
+        <v>148</v>
+      </c>
+      <c r="C787" t="n">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="n">
+        <v>45</v>
+      </c>
+      <c r="B788" t="n">
+        <v>436</v>
+      </c>
+      <c r="C788" t="n">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="n">
+        <v>46</v>
+      </c>
+      <c r="B789" t="n">
+        <v>261</v>
+      </c>
+      <c r="C789" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="n">
+        <v>47</v>
+      </c>
+      <c r="B790" t="n">
+        <v>441</v>
+      </c>
+      <c r="C790" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="n">
+        <v>48</v>
+      </c>
+      <c r="B791" t="n">
+        <v>430</v>
+      </c>
+      <c r="C791" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="n">
+        <v>49</v>
+      </c>
+      <c r="B792" t="n">
+        <v>333</v>
+      </c>
+      <c r="C792" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="n">
+        <v>50</v>
+      </c>
+      <c r="B793" t="n">
+        <v>106</v>
+      </c>
+      <c r="C793" t="n">
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Barycentre fix + enveloppe convex points + méthode bizzard de margherita qui marche à moitier (à fix)
flemme
</commit_message>
<xml_diff>
--- a/ListPoint.xlsx
+++ b/ListPoint.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuille1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>

</xml_diff>

<commit_message>
Mediane + fix deux trois truc
</commit_message>
<xml_diff>
--- a/ListPoint.xlsx
+++ b/ListPoint.xlsx
@@ -262,9 +262,615 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1" t="n">
+        <v>195</v>
+      </c>
+      <c r="C1" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="n">
+        <v>806</v>
+      </c>
+      <c r="C2" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="n">
+        <v>601</v>
+      </c>
+      <c r="C3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="n">
+        <v>552</v>
+      </c>
+      <c r="C4" t="n">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>701</v>
+      </c>
+      <c r="C5" t="n">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>787</v>
+      </c>
+      <c r="C6" t="n">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="n">
+        <v>913</v>
+      </c>
+      <c r="C7" t="n">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="n">
+        <v>552</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="n">
+        <v>674</v>
+      </c>
+      <c r="C9" t="n">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="n">
+        <v>992</v>
+      </c>
+      <c r="C10" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1065</v>
+      </c>
+      <c r="C11" t="n">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="n">
+        <v>801</v>
+      </c>
+      <c r="C12" t="n">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C13" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1095</v>
+      </c>
+      <c r="C14" t="n">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="n">
+        <v>534</v>
+      </c>
+      <c r="C15" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" t="n">
+        <v>90</v>
+      </c>
+      <c r="C16" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" t="n">
+        <v>722</v>
+      </c>
+      <c r="C17" t="n">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" t="n">
+        <v>495</v>
+      </c>
+      <c r="C18" t="n">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C19" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1182</v>
+      </c>
+      <c r="C20" t="n">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="n">
+        <v>878</v>
+      </c>
+      <c r="C21" t="n">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1074</v>
+      </c>
+      <c r="C22" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" t="n">
+        <v>689</v>
+      </c>
+      <c r="C23" t="n">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" t="n">
+        <v>853</v>
+      </c>
+      <c r="C24" t="n">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="n">
+        <v>836</v>
+      </c>
+      <c r="C25" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" t="n">
+        <v>12</v>
+      </c>
+      <c r="C26" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1155</v>
+      </c>
+      <c r="C27" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" t="n">
+        <v>313</v>
+      </c>
+      <c r="C28" t="n">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" t="n">
+        <v>667</v>
+      </c>
+      <c r="C29" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" t="n">
+        <v>378</v>
+      </c>
+      <c r="C30" t="n">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B31" t="n">
+        <v>706</v>
+      </c>
+      <c r="C31" t="n">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" t="n">
+        <v>771</v>
+      </c>
+      <c r="C32" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" t="n">
+        <v>977</v>
+      </c>
+      <c r="C33" t="n">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>7</v>
+      </c>
+      <c r="B34" t="n">
+        <v>400</v>
+      </c>
+      <c r="C34" t="n">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" t="n">
+        <v>442</v>
+      </c>
+      <c r="C35" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1073</v>
+      </c>
+      <c r="C36" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B37" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" t="n">
+        <v>43</v>
+      </c>
+      <c r="C38" t="n">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" t="n">
+        <v>610</v>
+      </c>
+      <c r="C39" t="n">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" t="n">
+        <v>47</v>
+      </c>
+      <c r="C40" t="n">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" t="n">
+        <v>231</v>
+      </c>
+      <c r="C41" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" t="n">
+        <v>806</v>
+      </c>
+      <c r="C42" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" t="n">
+        <v>708</v>
+      </c>
+      <c r="C43" t="n">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>3</v>
+      </c>
+      <c r="B44" t="n">
+        <v>732</v>
+      </c>
+      <c r="C44" t="n">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" t="n">
+        <v>529</v>
+      </c>
+      <c r="C45" t="n">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>5</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1195</v>
+      </c>
+      <c r="C46" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>6</v>
+      </c>
+      <c r="B47" t="n">
+        <v>26</v>
+      </c>
+      <c r="C47" t="n">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>7</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C48" t="n">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" t="n">
+        <v>405</v>
+      </c>
+      <c r="C49" t="n">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" t="n">
+        <v>261</v>
+      </c>
+      <c r="C50" t="n">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="n">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" t="n">
+        <v>744</v>
+      </c>
+      <c r="C52" t="n">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1038</v>
+      </c>
+      <c r="C53" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" t="n">
+        <v>383</v>
+      </c>
+      <c r="C54" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" t="n">
+        <v>954</v>
+      </c>
+      <c r="C55" t="n">
+        <v>363</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>